<commit_message>
Add new chat session and update session data
Add new chat session file data/user_sessions/ChatSessions/chat_session_20260615_112536_e4ed9973.json containing a user question about importing qualitative data and the assistant response. Update Data/user_sessions/session_metadata.json to register the new session and append a corresponding timed response to Data/user_sessions/timed_responses.json (response_time 11.05, timestamp 2026-06-15T10:25:47.804Z). Also update Data/evaluation/query_responses.xlsx (binary changes).
</commit_message>
<xml_diff>
--- a/Data/evaluation/query_responses.xlsx
+++ b/Data/evaluation/query_responses.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C343"/>
+  <dimension ref="A1:C344"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -6425,6 +6425,25 @@
         </is>
       </c>
     </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>How do I import qualitative data into GEO?</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>llama3.2:latest</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Option 1: Export to File; select Export to File, browse to a location, enter a file name, and select Save.
+Option 2: Export to Clipboard; select Export to Clipboard, open an external application (i.e. Excel), paste the contents of your clipboard.
+Option 3: Import from File; select Import from File, browse to the .txt file, select it, and Open.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>